<commit_message>
Add Aachen district clustering workflow
</commit_message>
<xml_diff>
--- a/districtgenerator/data/typdistrict_parameters.xlsx
+++ b/districtgenerator/data/typdistrict_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1B7C7C-4A1A-4D0B-B125-9EA3AA809974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C986DE7-23B0-422D-84F4-683E7AD7734A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16710" yWindow="-16395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16965" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -420,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -456,7 +456,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -480,6 +479,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -798,20 +803,20 @@
   <dimension ref="A1:AU11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="4" width="24.6640625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" style="19" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" style="19" customWidth="1"/>
-    <col min="10" max="10" width="16" style="19" customWidth="1"/>
-    <col min="11" max="11" width="14.33203125" style="19" customWidth="1"/>
-    <col min="12" max="12" width="14.5546875" style="19" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" style="19" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="19" customWidth="1"/>
-    <col min="15" max="15" width="15" style="19" customWidth="1"/>
-    <col min="38" max="39" width="17.33203125" style="19" customWidth="1"/>
-    <col min="40" max="40" width="17.109375" style="19" customWidth="1"/>
-    <col min="41" max="41" width="16.88671875" style="19" customWidth="1"/>
-    <col min="42" max="42" width="19" style="19" customWidth="1"/>
+    <col min="2" max="4" width="24.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14.5546875" customWidth="1"/>
+    <col min="13" max="13" width="18.6640625" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" customWidth="1"/>
+    <col min="15" max="15" width="15" customWidth="1"/>
+    <col min="38" max="39" width="17.33203125" customWidth="1"/>
+    <col min="40" max="40" width="17.109375" customWidth="1"/>
+    <col min="41" max="41" width="16.88671875" customWidth="1"/>
+    <col min="42" max="42" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:47" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -851,10 +856,10 @@
       <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="30" t="s">
         <v>13</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -905,13 +910,13 @@
       <c r="AE1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="23" t="s">
+      <c r="AF1" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="24" t="s">
+      <c r="AG1" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="25" t="s">
+      <c r="AH1" s="24" t="s">
         <v>32</v>
       </c>
       <c r="AI1" s="1" t="s">
@@ -1061,28 +1066,28 @@
       <c r="AI2" s="13">
         <v>10</v>
       </c>
-      <c r="AJ2" s="20">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="20">
+      <c r="AJ2" s="19">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="19">
         <v>20</v>
       </c>
-      <c r="AL2" s="20">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="20">
-        <v>0</v>
-      </c>
-      <c r="AN2" s="20">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="20">
+      <c r="AL2" s="19">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="19">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="19">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="19">
         <v>10</v>
       </c>
-      <c r="AP2" s="20">
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="20">
+      <c r="AP2" s="19">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="19">
         <v>20</v>
       </c>
       <c r="AR2" s="14">
@@ -1091,7 +1096,7 @@
       <c r="AS2" s="13">
         <v>7.3529411764705799</v>
       </c>
-      <c r="AT2" s="20">
+      <c r="AT2" s="19">
         <v>0</v>
       </c>
       <c r="AU2" s="14">
@@ -1205,28 +1210,28 @@
       <c r="AI3" s="13">
         <v>0</v>
       </c>
-      <c r="AJ3" s="20">
+      <c r="AJ3" s="19">
         <v>12.5</v>
       </c>
-      <c r="AK3" s="20">
+      <c r="AK3" s="19">
         <v>18.75</v>
       </c>
-      <c r="AL3" s="20">
+      <c r="AL3" s="19">
         <v>6.25</v>
       </c>
-      <c r="AM3" s="20">
-        <v>0</v>
-      </c>
-      <c r="AN3" s="20">
+      <c r="AM3" s="19">
+        <v>0</v>
+      </c>
+      <c r="AN3" s="19">
         <v>6.25</v>
       </c>
-      <c r="AO3" s="20">
+      <c r="AO3" s="19">
         <v>12.5</v>
       </c>
-      <c r="AP3" s="20">
+      <c r="AP3" s="19">
         <v>12.5</v>
       </c>
-      <c r="AQ3" s="20">
+      <c r="AQ3" s="19">
         <v>25</v>
       </c>
       <c r="AR3" s="14">
@@ -1235,7 +1240,7 @@
       <c r="AS3" s="13">
         <v>23.711340206185501</v>
       </c>
-      <c r="AT3" s="20">
+      <c r="AT3" s="19">
         <v>0</v>
       </c>
       <c r="AU3" s="14">
@@ -1349,28 +1354,28 @@
       <c r="AI4" s="13">
         <v>12.5</v>
       </c>
-      <c r="AJ4" s="20">
+      <c r="AJ4" s="19">
         <v>17.857142857142861</v>
       </c>
-      <c r="AK4" s="20">
+      <c r="AK4" s="19">
         <v>16.071428571428569</v>
       </c>
-      <c r="AL4" s="20">
+      <c r="AL4" s="19">
         <v>12.5</v>
       </c>
-      <c r="AM4" s="20">
-        <v>0</v>
-      </c>
-      <c r="AN4" s="20">
+      <c r="AM4" s="19">
+        <v>0</v>
+      </c>
+      <c r="AN4" s="19">
         <v>3.5714285714285721</v>
       </c>
-      <c r="AO4" s="20">
+      <c r="AO4" s="19">
         <v>5.3571428571428568</v>
       </c>
-      <c r="AP4" s="20">
+      <c r="AP4" s="19">
         <v>8.9285714285714288</v>
       </c>
-      <c r="AQ4" s="20">
+      <c r="AQ4" s="19">
         <v>7.1428571428571432</v>
       </c>
       <c r="AR4" s="14">
@@ -1379,7 +1384,7 @@
       <c r="AS4" s="13">
         <v>6.59945004582951</v>
       </c>
-      <c r="AT4" s="20">
+      <c r="AT4" s="19">
         <v>1.1915673693858799</v>
       </c>
       <c r="AU4" s="14">
@@ -1493,28 +1498,28 @@
       <c r="AI5" s="13">
         <v>15.38461538461539</v>
       </c>
-      <c r="AJ5" s="20">
+      <c r="AJ5" s="19">
         <v>22.37762237762238</v>
       </c>
-      <c r="AK5" s="20">
+      <c r="AK5" s="19">
         <v>13.98601398601399</v>
       </c>
-      <c r="AL5" s="20">
+      <c r="AL5" s="19">
         <v>6.2937062937062933</v>
       </c>
-      <c r="AM5" s="20">
-        <v>0</v>
-      </c>
-      <c r="AN5" s="20">
+      <c r="AM5" s="19">
+        <v>0</v>
+      </c>
+      <c r="AN5" s="19">
         <v>18.18181818181818</v>
       </c>
-      <c r="AO5" s="20">
+      <c r="AO5" s="19">
         <v>0.69930069930069927</v>
       </c>
-      <c r="AP5" s="20">
+      <c r="AP5" s="19">
         <v>4.895104895104895</v>
       </c>
-      <c r="AQ5" s="20">
+      <c r="AQ5" s="19">
         <v>14.68531468531468</v>
       </c>
       <c r="AR5" s="14">
@@ -1523,7 +1528,7 @@
       <c r="AS5" s="13">
         <v>1.4891179839633399</v>
       </c>
-      <c r="AT5" s="20">
+      <c r="AT5" s="19">
         <v>0.39455262822960402</v>
       </c>
       <c r="AU5" s="14">
@@ -1637,28 +1642,28 @@
       <c r="AI6" s="13">
         <v>8.125</v>
       </c>
-      <c r="AJ6" s="20">
+      <c r="AJ6" s="19">
         <v>11.77083333333333</v>
       </c>
-      <c r="AK6" s="20">
+      <c r="AK6" s="19">
         <v>17.291666666666671</v>
       </c>
-      <c r="AL6" s="20">
+      <c r="AL6" s="19">
         <v>7.916666666666667</v>
       </c>
-      <c r="AM6" s="20">
+      <c r="AM6" s="19">
         <v>0.1041666666666667</v>
       </c>
-      <c r="AN6" s="20">
+      <c r="AN6" s="19">
         <v>10.3125</v>
       </c>
-      <c r="AO6" s="20">
+      <c r="AO6" s="19">
         <v>3.645833333333333</v>
       </c>
-      <c r="AP6" s="20">
+      <c r="AP6" s="19">
         <v>2.083333333333333</v>
       </c>
-      <c r="AQ6" s="20">
+      <c r="AQ6" s="19">
         <v>30.9375</v>
       </c>
       <c r="AR6" s="14">
@@ -1667,7 +1672,7 @@
       <c r="AS6" s="13">
         <v>2.6750869225856801</v>
       </c>
-      <c r="AT6" s="20">
+      <c r="AT6" s="19">
         <v>4.3212942595614798</v>
       </c>
       <c r="AU6" s="14">
@@ -1781,28 +1786,28 @@
       <c r="AI7" s="13">
         <v>9.6256684491978604</v>
       </c>
-      <c r="AJ7" s="20">
+      <c r="AJ7" s="19">
         <v>18.71657754010695</v>
       </c>
-      <c r="AK7" s="20">
+      <c r="AK7" s="19">
         <v>16.042780748663102</v>
       </c>
-      <c r="AL7" s="20">
+      <c r="AL7" s="19">
         <v>7.4866310160427796</v>
       </c>
-      <c r="AM7" s="20">
-        <v>0</v>
-      </c>
-      <c r="AN7" s="20">
+      <c r="AM7" s="19">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="19">
         <v>12.834224598930479</v>
       </c>
-      <c r="AO7" s="20">
+      <c r="AO7" s="19">
         <v>2.1390374331550799</v>
       </c>
-      <c r="AP7" s="20">
+      <c r="AP7" s="19">
         <v>2.1390374331550799</v>
       </c>
-      <c r="AQ7" s="20">
+      <c r="AQ7" s="19">
         <v>26.203208556149729</v>
       </c>
       <c r="AR7" s="14">
@@ -1811,7 +1816,7 @@
       <c r="AS7" s="13">
         <v>4.5631411390166203</v>
       </c>
-      <c r="AT7" s="20">
+      <c r="AT7" s="19">
         <v>2.2285107888220699</v>
       </c>
       <c r="AU7" s="14">
@@ -1925,28 +1930,28 @@
       <c r="AI8" s="13">
         <v>5.2708638360175692</v>
       </c>
-      <c r="AJ8" s="20">
+      <c r="AJ8" s="19">
         <v>34.407027818448022</v>
       </c>
-      <c r="AK8" s="20">
+      <c r="AK8" s="19">
         <v>9.3704245973645683</v>
       </c>
-      <c r="AL8" s="20">
+      <c r="AL8" s="19">
         <v>9.9560761346998543</v>
       </c>
-      <c r="AM8" s="20">
+      <c r="AM8" s="19">
         <v>1.171303074670571</v>
       </c>
-      <c r="AN8" s="20">
+      <c r="AN8" s="19">
         <v>13.909224011713031</v>
       </c>
-      <c r="AO8" s="20">
+      <c r="AO8" s="19">
         <v>5.1244509516837482</v>
       </c>
-      <c r="AP8" s="20">
+      <c r="AP8" s="19">
         <v>6.5885797950219622</v>
       </c>
-      <c r="AQ8" s="20">
+      <c r="AQ8" s="19">
         <v>11.859443631039531</v>
       </c>
       <c r="AR8" s="14">
@@ -1955,7 +1960,7 @@
       <c r="AS8" s="13">
         <v>11.3055902839792</v>
       </c>
-      <c r="AT8" s="20">
+      <c r="AT8" s="19">
         <v>1.75031255581353</v>
       </c>
       <c r="AU8" s="14">
@@ -2069,28 +2074,28 @@
       <c r="AI9" s="13">
         <v>11.060339777387229</v>
       </c>
-      <c r="AJ9" s="20">
+      <c r="AJ9" s="19">
         <v>6.4674868189806682</v>
       </c>
-      <c r="AK9" s="20">
+      <c r="AK9" s="19">
         <v>24.42882249560633</v>
       </c>
-      <c r="AL9" s="20">
+      <c r="AL9" s="19">
         <v>7.2056239015817223</v>
       </c>
-      <c r="AM9" s="20">
+      <c r="AM9" s="19">
         <v>1.7106033977738719</v>
       </c>
-      <c r="AN9" s="20">
+      <c r="AN9" s="19">
         <v>12.00937316930287</v>
       </c>
-      <c r="AO9" s="20">
+      <c r="AO9" s="19">
         <v>2.9759812536613941</v>
       </c>
-      <c r="AP9" s="20">
+      <c r="AP9" s="19">
         <v>2.1792618629173992</v>
       </c>
-      <c r="AQ9" s="20">
+      <c r="AQ9" s="19">
         <v>27.00644405389572</v>
       </c>
       <c r="AR9" s="14">
@@ -2099,7 +2104,7 @@
       <c r="AS9" s="13">
         <v>9.7592553712646097</v>
       </c>
-      <c r="AT9" s="20">
+      <c r="AT9" s="19">
         <v>20.634754006578401</v>
       </c>
       <c r="AU9" s="14">
@@ -2113,10 +2118,10 @@
       <c r="B10" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="20">
         <v>1.5</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="21">
         <v>4.5</v>
       </c>
       <c r="E10" s="3">
@@ -2254,57 +2259,57 @@
       <c r="A11" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="28"/>
-      <c r="S11" s="26" t="s">
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
+      <c r="N11" s="26"/>
+      <c r="O11" s="26"/>
+      <c r="P11" s="26"/>
+      <c r="Q11" s="26"/>
+      <c r="R11" s="27"/>
+      <c r="S11" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="T11" s="27"/>
-      <c r="U11" s="27"/>
-      <c r="V11" s="27"/>
-      <c r="W11" s="27"/>
-      <c r="X11" s="27"/>
-      <c r="Y11" s="27"/>
-      <c r="Z11" s="27"/>
-      <c r="AA11" s="27"/>
-      <c r="AB11" s="28"/>
-      <c r="AC11" s="26" t="s">
+      <c r="T11" s="26"/>
+      <c r="U11" s="26"/>
+      <c r="V11" s="26"/>
+      <c r="W11" s="26"/>
+      <c r="X11" s="26"/>
+      <c r="Y11" s="26"/>
+      <c r="Z11" s="26"/>
+      <c r="AA11" s="26"/>
+      <c r="AB11" s="27"/>
+      <c r="AC11" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="AD11" s="27"/>
-      <c r="AE11" s="28"/>
-      <c r="AF11" s="26" t="s">
+      <c r="AD11" s="26"/>
+      <c r="AE11" s="27"/>
+      <c r="AF11" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="AG11" s="27"/>
-      <c r="AH11" s="28"/>
-      <c r="AI11" s="20"/>
-      <c r="AJ11" s="20"/>
-      <c r="AK11" s="20"/>
-      <c r="AL11" s="20"/>
-      <c r="AM11" s="20"/>
-      <c r="AN11" s="20"/>
-      <c r="AO11" s="20"/>
-      <c r="AP11" s="20"/>
-      <c r="AQ11" s="20"/>
-      <c r="AR11" s="20"/>
+      <c r="AG11" s="26"/>
+      <c r="AH11" s="27"/>
+      <c r="AI11" s="19"/>
+      <c r="AJ11" s="19"/>
+      <c r="AK11" s="19"/>
+      <c r="AL11" s="19"/>
+      <c r="AM11" s="19"/>
+      <c r="AN11" s="19"/>
+      <c r="AO11" s="19"/>
+      <c r="AP11" s="19"/>
+      <c r="AQ11" s="19"/>
+      <c r="AR11" s="19"/>
       <c r="AS11" s="18"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update typdistrict parameters with OSM results
</commit_message>
<xml_diff>
--- a/districtgenerator/data/typdistrict_parameters.xlsx
+++ b/districtgenerator/data/typdistrict_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C986DE7-23B0-422D-84F4-683E7AD7734A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1B40B7-3F48-4730-BEFC-79E6ED7F369D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16965" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11835" yWindow="-16335" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -420,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -479,12 +479,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,10 +850,10 @@
       <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="29" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="30" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -1064,16 +1058,16 @@
         <v>3.5</v>
       </c>
       <c r="AI2" s="13">
-        <v>10</v>
+        <v>32.14</v>
       </c>
       <c r="AJ2" s="19">
         <v>0</v>
       </c>
       <c r="AK2" s="19">
-        <v>20</v>
+        <v>10.71</v>
       </c>
       <c r="AL2" s="19">
-        <v>0</v>
+        <v>3.57</v>
       </c>
       <c r="AM2" s="19">
         <v>0</v>
@@ -1082,25 +1076,25 @@
         <v>0</v>
       </c>
       <c r="AO2" s="19">
-        <v>10</v>
+        <v>10.71</v>
       </c>
       <c r="AP2" s="19">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="AQ2" s="19">
-        <v>20</v>
+        <v>10.71</v>
       </c>
       <c r="AR2" s="14">
-        <v>40</v>
+        <v>7.14</v>
       </c>
       <c r="AS2" s="13">
-        <v>7.3529411764705799</v>
+        <v>50.59</v>
       </c>
       <c r="AT2" s="19">
         <v>0</v>
       </c>
       <c r="AU2" s="14">
-        <v>92.647058823529406</v>
+        <v>49.41</v>
       </c>
     </row>
     <row r="3" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1208,43 +1202,43 @@
         <v>3</v>
       </c>
       <c r="AI3" s="13">
-        <v>0</v>
+        <v>12.6</v>
       </c>
       <c r="AJ3" s="19">
-        <v>12.5</v>
+        <v>9.4499999999999993</v>
       </c>
       <c r="AK3" s="19">
-        <v>18.75</v>
+        <v>11.81</v>
       </c>
       <c r="AL3" s="19">
-        <v>6.25</v>
+        <v>7.87</v>
       </c>
       <c r="AM3" s="19">
         <v>0</v>
       </c>
       <c r="AN3" s="19">
-        <v>6.25</v>
+        <v>1.57</v>
       </c>
       <c r="AO3" s="19">
-        <v>12.5</v>
+        <v>3.15</v>
       </c>
       <c r="AP3" s="19">
-        <v>12.5</v>
+        <v>10.24</v>
       </c>
       <c r="AQ3" s="19">
-        <v>25</v>
+        <v>20.47</v>
       </c>
       <c r="AR3" s="14">
-        <v>6.25</v>
+        <v>22.83</v>
       </c>
       <c r="AS3" s="13">
-        <v>23.711340206185501</v>
+        <v>11.03</v>
       </c>
       <c r="AT3" s="19">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="AU3" s="14">
-        <v>76.288659793814404</v>
+        <v>88.02</v>
       </c>
     </row>
     <row r="4" spans="1:47" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1352,43 +1346,43 @@
         <v>3.5</v>
       </c>
       <c r="AI4" s="13">
-        <v>12.5</v>
+        <v>8.11</v>
       </c>
       <c r="AJ4" s="19">
-        <v>17.857142857142861</v>
+        <v>16.760000000000002</v>
       </c>
       <c r="AK4" s="19">
-        <v>16.071428571428569</v>
+        <v>7.03</v>
       </c>
       <c r="AL4" s="19">
-        <v>12.5</v>
+        <v>5.95</v>
       </c>
       <c r="AM4" s="19">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="AN4" s="19">
-        <v>3.5714285714285721</v>
+        <v>4.32</v>
       </c>
       <c r="AO4" s="19">
-        <v>5.3571428571428568</v>
+        <v>3.78</v>
       </c>
       <c r="AP4" s="19">
-        <v>8.9285714285714288</v>
+        <v>7.03</v>
       </c>
       <c r="AQ4" s="19">
-        <v>7.1428571428571432</v>
+        <v>21.08</v>
       </c>
       <c r="AR4" s="14">
-        <v>16.071428571428569</v>
+        <v>24.86</v>
       </c>
       <c r="AS4" s="13">
-        <v>6.59945004582951</v>
+        <v>25.9</v>
       </c>
       <c r="AT4" s="19">
-        <v>1.1915673693858799</v>
+        <v>1.08</v>
       </c>
       <c r="AU4" s="14">
-        <v>92.208982584784593</v>
+        <v>73.03</v>
       </c>
     </row>
     <row r="5" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1496,43 +1490,43 @@
         <v>3.5</v>
       </c>
       <c r="AI5" s="13">
-        <v>15.38461538461539</v>
+        <v>9.39</v>
       </c>
       <c r="AJ5" s="19">
-        <v>22.37762237762238</v>
+        <v>14.56</v>
       </c>
       <c r="AK5" s="19">
-        <v>13.98601398601399</v>
+        <v>9</v>
       </c>
       <c r="AL5" s="19">
-        <v>6.2937062937062933</v>
+        <v>5.36</v>
       </c>
       <c r="AM5" s="19">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="AN5" s="19">
-        <v>18.18181818181818</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="AO5" s="19">
-        <v>0.69930069930069927</v>
+        <v>2.68</v>
       </c>
       <c r="AP5" s="19">
-        <v>4.895104895104895</v>
+        <v>4.9800000000000004</v>
       </c>
       <c r="AQ5" s="19">
-        <v>14.68531468531468</v>
+        <v>22.22</v>
       </c>
       <c r="AR5" s="14">
-        <v>3.4965034965034971</v>
+        <v>21.46</v>
       </c>
       <c r="AS5" s="13">
-        <v>1.4891179839633399</v>
+        <v>22.12</v>
       </c>
       <c r="AT5" s="19">
-        <v>0.39455262822960402</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AU5" s="14">
-        <v>98.116329387806999</v>
+        <v>76.78</v>
       </c>
     </row>
     <row r="6" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1640,43 +1634,43 @@
         <v>3</v>
       </c>
       <c r="AI6" s="13">
-        <v>8.125</v>
+        <v>5.82</v>
       </c>
       <c r="AJ6" s="19">
-        <v>11.77083333333333</v>
+        <v>17.77</v>
       </c>
       <c r="AK6" s="19">
-        <v>17.291666666666671</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="AL6" s="19">
-        <v>7.916666666666667</v>
+        <v>8.02</v>
       </c>
       <c r="AM6" s="19">
-        <v>0.1041666666666667</v>
+        <v>0</v>
       </c>
       <c r="AN6" s="19">
-        <v>10.3125</v>
+        <v>7.7</v>
       </c>
       <c r="AO6" s="19">
-        <v>3.645833333333333</v>
+        <v>2.36</v>
       </c>
       <c r="AP6" s="19">
-        <v>2.083333333333333</v>
+        <v>2.36</v>
       </c>
       <c r="AQ6" s="19">
-        <v>30.9375</v>
+        <v>25.16</v>
       </c>
       <c r="AR6" s="14">
-        <v>7.8125</v>
+        <v>12.42</v>
       </c>
       <c r="AS6" s="13">
-        <v>2.6750869225856801</v>
+        <v>6.45</v>
       </c>
       <c r="AT6" s="19">
-        <v>4.3212942595614798</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="AU6" s="14">
-        <v>93.003618817852796</v>
+        <v>92.98</v>
       </c>
     </row>
     <row r="7" spans="1:47" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1784,43 +1778,43 @@
         <v>6</v>
       </c>
       <c r="AI7" s="13">
-        <v>9.6256684491978604</v>
+        <v>0</v>
       </c>
       <c r="AJ7" s="19">
-        <v>18.71657754010695</v>
+        <v>0</v>
       </c>
       <c r="AK7" s="19">
-        <v>16.042780748663102</v>
+        <v>16.670000000000002</v>
       </c>
       <c r="AL7" s="19">
-        <v>7.4866310160427796</v>
+        <v>0</v>
       </c>
       <c r="AM7" s="19">
         <v>0</v>
       </c>
       <c r="AN7" s="19">
-        <v>12.834224598930479</v>
+        <v>0</v>
       </c>
       <c r="AO7" s="19">
-        <v>2.1390374331550799</v>
+        <v>0</v>
       </c>
       <c r="AP7" s="19">
-        <v>2.1390374331550799</v>
+        <v>0</v>
       </c>
       <c r="AQ7" s="19">
-        <v>26.203208556149729</v>
+        <v>33.33</v>
       </c>
       <c r="AR7" s="14">
-        <v>4.8128342245989302</v>
+        <v>50</v>
       </c>
       <c r="AS7" s="13">
-        <v>4.5631411390166203</v>
+        <v>22.86</v>
       </c>
       <c r="AT7" s="19">
-        <v>2.2285107888220699</v>
+        <v>0</v>
       </c>
       <c r="AU7" s="14">
-        <v>93.2083480721613</v>
+        <v>77.14</v>
       </c>
     </row>
     <row r="8" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1928,43 +1922,43 @@
         <v>19</v>
       </c>
       <c r="AI8" s="13">
-        <v>5.2708638360175692</v>
+        <v>10.53</v>
       </c>
       <c r="AJ8" s="19">
-        <v>34.407027818448022</v>
+        <v>19.62</v>
       </c>
       <c r="AK8" s="19">
-        <v>9.3704245973645683</v>
+        <v>7.18</v>
       </c>
       <c r="AL8" s="19">
-        <v>9.9560761346998543</v>
+        <v>2.87</v>
       </c>
       <c r="AM8" s="19">
-        <v>1.171303074670571</v>
+        <v>12.44</v>
       </c>
       <c r="AN8" s="19">
-        <v>13.909224011713031</v>
+        <v>5.26</v>
       </c>
       <c r="AO8" s="19">
-        <v>5.1244509516837482</v>
+        <v>2.39</v>
       </c>
       <c r="AP8" s="19">
-        <v>6.5885797950219622</v>
+        <v>6.7</v>
       </c>
       <c r="AQ8" s="19">
-        <v>11.859443631039531</v>
+        <v>12.44</v>
       </c>
       <c r="AR8" s="14">
-        <v>2.3426061493411421</v>
+        <v>20.57</v>
       </c>
       <c r="AS8" s="13">
-        <v>11.3055902839792</v>
+        <v>30.38</v>
       </c>
       <c r="AT8" s="19">
-        <v>1.75031255581353</v>
+        <v>2.69</v>
       </c>
       <c r="AU8" s="14">
-        <v>86.944097160207093</v>
+        <v>66.92</v>
       </c>
     </row>
     <row r="9" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2072,43 +2066,43 @@
         <v>6</v>
       </c>
       <c r="AI9" s="13">
-        <v>11.060339777387229</v>
+        <v>16.05</v>
       </c>
       <c r="AJ9" s="19">
-        <v>6.4674868189806682</v>
+        <v>14.72</v>
       </c>
       <c r="AK9" s="19">
-        <v>24.42882249560633</v>
+        <v>9.0299999999999994</v>
       </c>
       <c r="AL9" s="19">
-        <v>7.2056239015817223</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="AM9" s="19">
-        <v>1.7106033977738719</v>
+        <v>7.36</v>
       </c>
       <c r="AN9" s="19">
-        <v>12.00937316930287</v>
+        <v>10.029999999999999</v>
       </c>
       <c r="AO9" s="19">
-        <v>2.9759812536613941</v>
+        <v>1.67</v>
       </c>
       <c r="AP9" s="19">
-        <v>2.1792618629173992</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="AQ9" s="19">
-        <v>27.00644405389572</v>
+        <v>24.75</v>
       </c>
       <c r="AR9" s="14">
-        <v>4.9560632688927946</v>
+        <v>7.02</v>
       </c>
       <c r="AS9" s="13">
-        <v>9.7592553712646097</v>
+        <v>19.95</v>
       </c>
       <c r="AT9" s="19">
-        <v>20.634754006578401</v>
+        <v>7.91</v>
       </c>
       <c r="AU9" s="14">
-        <v>69.605990622156895</v>
+        <v>72.14</v>
       </c>
     </row>
     <row r="10" spans="1:47" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2216,43 +2210,43 @@
         <v>6.5</v>
       </c>
       <c r="AI10" s="15">
-        <v>12.34163795388285</v>
+        <v>10.45</v>
       </c>
       <c r="AJ10" s="16">
-        <v>3.339517625231911</v>
+        <v>3.78</v>
       </c>
       <c r="AK10" s="16">
-        <v>25.815001325205412</v>
+        <v>20.18</v>
       </c>
       <c r="AL10" s="16">
-        <v>4.7707394646170158</v>
+        <v>7.93</v>
       </c>
       <c r="AM10" s="16">
-        <v>2.517890272992314</v>
+        <v>1.8</v>
       </c>
       <c r="AN10" s="16">
-        <v>6.3344818446859259</v>
+        <v>5.41</v>
       </c>
       <c r="AO10" s="16">
-        <v>4.1611449774715084</v>
+        <v>1.98</v>
       </c>
       <c r="AP10" s="16">
-        <v>0.76861913596607478</v>
+        <v>1.26</v>
       </c>
       <c r="AQ10" s="16">
-        <v>35.849986747945927</v>
+        <v>41.98</v>
       </c>
       <c r="AR10" s="17">
-        <v>4.1009806520010601</v>
+        <v>5.23</v>
       </c>
       <c r="AS10" s="15">
-        <v>23.565676899848999</v>
+        <v>12.41</v>
       </c>
       <c r="AT10" s="16">
-        <v>24.408656265727199</v>
+        <v>13.38</v>
       </c>
       <c r="AU10" s="17">
-        <v>52.025666834423703</v>
+        <v>74.209999999999994</v>
       </c>
     </row>
     <row r="11" spans="1:47" ht="105" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Integrate corrected OSM use probabilities into the existing workflow
</commit_message>
<xml_diff>
--- a/districtgenerator/data/typdistrict_parameters.xlsx
+++ b/districtgenerator/data/typdistrict_parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1B40B7-3F48-4730-BEFC-79E6ED7F369D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B0F1B52-63FF-4FBF-B32B-00B08FFE0E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11835" yWindow="-16335" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -176,6 +176,9 @@
     <t>A</t>
   </si>
   <si>
+    <t>Streusiedlungen</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
@@ -185,9 +188,15 @@
     <t>C</t>
   </si>
   <si>
+    <t>Wohnbebauung niedriger Dichte</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
+    <t>Wohnbebauung mittlerer Dichte</t>
+  </si>
+  <si>
     <t>E</t>
   </si>
   <si>
@@ -213,6 +222,9 @@
   </si>
   <si>
     <t>I</t>
+  </si>
+  <si>
+    <t>Innenstadt</t>
   </si>
   <si>
     <t>Quelle:</t>
@@ -238,18 +250,6 @@
 energetische Kennwerte von Stadträumen. 2.,
 überarb. und erw. Aufl. Stuttgart: Fraunhofer IRB
 Verlag.</t>
-  </si>
-  <si>
-    <t>Wohnbebauung niedriger Dichte</t>
-  </si>
-  <si>
-    <t>Wohnbebauung mittlerer Dichte</t>
-  </si>
-  <si>
-    <t>Streusiedlungen</t>
-  </si>
-  <si>
-    <t>Innenstadt</t>
   </si>
 </sst>
 </file>
@@ -540,7 +540,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -592,7 +592,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -653,23 +653,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -679,23 +679,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -703,26 +703,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -757,17 +754,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -784,11 +781,6 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -798,7 +790,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="4" width="24.6640625" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
@@ -958,7 +950,7 @@
         <v>46</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="C2" s="3">
         <v>2.5000000000000001E-2</v>
@@ -1058,16 +1050,16 @@
         <v>3.5</v>
       </c>
       <c r="AI2" s="13">
-        <v>32.14</v>
+        <v>40.909999999999997</v>
       </c>
       <c r="AJ2" s="19">
         <v>0</v>
       </c>
       <c r="AK2" s="19">
-        <v>10.71</v>
+        <v>13.64</v>
       </c>
       <c r="AL2" s="19">
-        <v>3.57</v>
+        <v>4.55</v>
       </c>
       <c r="AM2" s="19">
         <v>0</v>
@@ -1076,33 +1068,33 @@
         <v>0</v>
       </c>
       <c r="AO2" s="19">
-        <v>10.71</v>
+        <v>13.64</v>
       </c>
       <c r="AP2" s="19">
-        <v>25</v>
+        <v>4.55</v>
       </c>
       <c r="AQ2" s="19">
-        <v>10.71</v>
+        <v>13.64</v>
       </c>
       <c r="AR2" s="14">
-        <v>7.14</v>
+        <v>9.09</v>
       </c>
       <c r="AS2" s="13">
-        <v>50.59</v>
+        <v>13.21</v>
       </c>
       <c r="AT2" s="19">
         <v>0</v>
       </c>
       <c r="AU2" s="14">
-        <v>49.41</v>
+        <v>86.79</v>
       </c>
     </row>
     <row r="3" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3">
         <v>0.05</v>
@@ -1202,51 +1194,51 @@
         <v>3</v>
       </c>
       <c r="AI3" s="13">
-        <v>12.6</v>
+        <v>13.56</v>
       </c>
       <c r="AJ3" s="19">
-        <v>9.4499999999999993</v>
+        <v>10.17</v>
       </c>
       <c r="AK3" s="19">
-        <v>11.81</v>
+        <v>12.71</v>
       </c>
       <c r="AL3" s="19">
-        <v>7.87</v>
+        <v>8.4700000000000006</v>
       </c>
       <c r="AM3" s="19">
         <v>0</v>
       </c>
       <c r="AN3" s="19">
-        <v>1.57</v>
+        <v>1.69</v>
       </c>
       <c r="AO3" s="19">
-        <v>3.15</v>
+        <v>3.39</v>
       </c>
       <c r="AP3" s="19">
-        <v>10.24</v>
+        <v>3.39</v>
       </c>
       <c r="AQ3" s="19">
-        <v>20.47</v>
+        <v>22.03</v>
       </c>
       <c r="AR3" s="14">
-        <v>22.83</v>
+        <v>24.58</v>
       </c>
       <c r="AS3" s="13">
-        <v>11.03</v>
+        <v>10.91</v>
       </c>
       <c r="AT3" s="19">
         <v>0.95</v>
       </c>
       <c r="AU3" s="14">
-        <v>88.02</v>
+        <v>88.15</v>
       </c>
     </row>
     <row r="4" spans="1:47" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C4" s="3">
         <v>0.05</v>
@@ -1346,51 +1338,51 @@
         <v>3.5</v>
       </c>
       <c r="AI4" s="13">
-        <v>8.11</v>
+        <v>8.57</v>
       </c>
       <c r="AJ4" s="19">
-        <v>16.760000000000002</v>
+        <v>17.71</v>
       </c>
       <c r="AK4" s="19">
-        <v>7.03</v>
+        <v>7.43</v>
       </c>
       <c r="AL4" s="19">
-        <v>5.95</v>
+        <v>6.29</v>
       </c>
       <c r="AM4" s="19">
-        <v>1.08</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="AN4" s="19">
-        <v>4.32</v>
+        <v>4.57</v>
       </c>
       <c r="AO4" s="19">
-        <v>3.78</v>
+        <v>4</v>
       </c>
       <c r="AP4" s="19">
-        <v>7.03</v>
+        <v>1.71</v>
       </c>
       <c r="AQ4" s="19">
-        <v>21.08</v>
+        <v>22.29</v>
       </c>
       <c r="AR4" s="14">
-        <v>24.86</v>
+        <v>26.29</v>
       </c>
       <c r="AS4" s="13">
-        <v>25.9</v>
+        <v>25.76</v>
       </c>
       <c r="AT4" s="19">
         <v>1.08</v>
       </c>
       <c r="AU4" s="14">
-        <v>73.03</v>
+        <v>73.16</v>
       </c>
     </row>
     <row r="5" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C5" s="3">
         <v>0.2</v>
@@ -1490,51 +1482,51 @@
         <v>3.5</v>
       </c>
       <c r="AI5" s="13">
-        <v>9.39</v>
+        <v>9.84</v>
       </c>
       <c r="AJ5" s="19">
-        <v>14.56</v>
+        <v>15.26</v>
       </c>
       <c r="AK5" s="19">
-        <v>9</v>
+        <v>9.44</v>
       </c>
       <c r="AL5" s="19">
-        <v>5.36</v>
+        <v>5.62</v>
       </c>
       <c r="AM5" s="19">
-        <v>6.32</v>
+        <v>6.63</v>
       </c>
       <c r="AN5" s="19">
-        <v>4.0199999999999996</v>
+        <v>4.22</v>
       </c>
       <c r="AO5" s="19">
-        <v>2.68</v>
+        <v>2.81</v>
       </c>
       <c r="AP5" s="19">
-        <v>4.9800000000000004</v>
+        <v>0.2</v>
       </c>
       <c r="AQ5" s="19">
-        <v>22.22</v>
+        <v>23.49</v>
       </c>
       <c r="AR5" s="14">
-        <v>21.46</v>
+        <v>22.49</v>
       </c>
       <c r="AS5" s="13">
-        <v>22.12</v>
+        <v>22.09</v>
       </c>
       <c r="AT5" s="19">
         <v>1.1000000000000001</v>
       </c>
       <c r="AU5" s="14">
-        <v>76.78</v>
+        <v>76.8</v>
       </c>
     </row>
     <row r="6" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C6" s="3">
         <v>0.2</v>
@@ -1634,51 +1626,51 @@
         <v>3</v>
       </c>
       <c r="AI6" s="13">
-        <v>5.82</v>
+        <v>5.88</v>
       </c>
       <c r="AJ6" s="19">
-        <v>17.77</v>
+        <v>17.97</v>
       </c>
       <c r="AK6" s="19">
-        <v>18.399999999999999</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="AL6" s="19">
-        <v>8.02</v>
+        <v>8.11</v>
       </c>
       <c r="AM6" s="19">
         <v>0</v>
       </c>
       <c r="AN6" s="19">
-        <v>7.7</v>
+        <v>7.79</v>
       </c>
       <c r="AO6" s="19">
-        <v>2.36</v>
+        <v>2.38</v>
       </c>
       <c r="AP6" s="19">
-        <v>2.36</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="AQ6" s="19">
-        <v>25.16</v>
+        <v>25.6</v>
       </c>
       <c r="AR6" s="14">
-        <v>12.42</v>
+        <v>12.56</v>
       </c>
       <c r="AS6" s="13">
-        <v>6.45</v>
+        <v>6.43</v>
       </c>
       <c r="AT6" s="19">
         <v>0.56999999999999995</v>
       </c>
       <c r="AU6" s="14">
-        <v>92.98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:47" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C7" s="3">
         <v>0.4</v>
@@ -1819,10 +1811,10 @@
     </row>
     <row r="8" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C8" s="3">
         <v>0.8</v>
@@ -1922,51 +1914,51 @@
         <v>19</v>
       </c>
       <c r="AI8" s="13">
-        <v>10.53</v>
+        <v>11.39</v>
       </c>
       <c r="AJ8" s="19">
-        <v>19.62</v>
+        <v>20.3</v>
       </c>
       <c r="AK8" s="19">
-        <v>7.18</v>
+        <v>7.43</v>
       </c>
       <c r="AL8" s="19">
-        <v>2.87</v>
+        <v>2.97</v>
       </c>
       <c r="AM8" s="19">
-        <v>12.44</v>
+        <v>12.87</v>
       </c>
       <c r="AN8" s="19">
-        <v>5.26</v>
+        <v>5.45</v>
       </c>
       <c r="AO8" s="19">
-        <v>2.39</v>
+        <v>2.48</v>
       </c>
       <c r="AP8" s="19">
-        <v>6.7</v>
+        <v>2.97</v>
       </c>
       <c r="AQ8" s="19">
-        <v>12.44</v>
+        <v>12.87</v>
       </c>
       <c r="AR8" s="14">
-        <v>20.57</v>
+        <v>21.29</v>
       </c>
       <c r="AS8" s="13">
-        <v>30.38</v>
+        <v>30.3</v>
       </c>
       <c r="AT8" s="19">
-        <v>2.69</v>
+        <v>2.7</v>
       </c>
       <c r="AU8" s="14">
-        <v>66.92</v>
+        <v>67.010000000000005</v>
       </c>
     </row>
     <row r="9" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C9" s="3">
         <v>0.5</v>
@@ -2066,51 +2058,51 @@
         <v>6</v>
       </c>
       <c r="AI9" s="13">
-        <v>16.05</v>
+        <v>16.27</v>
       </c>
       <c r="AJ9" s="19">
-        <v>14.72</v>
+        <v>14.92</v>
       </c>
       <c r="AK9" s="19">
-        <v>9.0299999999999994</v>
+        <v>9.15</v>
       </c>
       <c r="AL9" s="19">
-        <v>5.0199999999999996</v>
+        <v>5.08</v>
       </c>
       <c r="AM9" s="19">
-        <v>7.36</v>
+        <v>7.46</v>
       </c>
       <c r="AN9" s="19">
-        <v>10.029999999999999</v>
+        <v>10.17</v>
       </c>
       <c r="AO9" s="19">
-        <v>1.67</v>
+        <v>1.69</v>
       </c>
       <c r="AP9" s="19">
-        <v>4.3499999999999996</v>
+        <v>3.05</v>
       </c>
       <c r="AQ9" s="19">
-        <v>24.75</v>
+        <v>25.08</v>
       </c>
       <c r="AR9" s="14">
-        <v>7.02</v>
+        <v>7.12</v>
       </c>
       <c r="AS9" s="13">
-        <v>19.95</v>
+        <v>19.88</v>
       </c>
       <c r="AT9" s="19">
-        <v>7.91</v>
+        <v>7.92</v>
       </c>
       <c r="AU9" s="14">
-        <v>72.14</v>
+        <v>72.2</v>
       </c>
     </row>
-    <row r="10" spans="1:47" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C10" s="20">
         <v>1.5</v>
@@ -2210,34 +2202,34 @@
         <v>6.5</v>
       </c>
       <c r="AI10" s="15">
-        <v>10.45</v>
+        <v>10.53</v>
       </c>
       <c r="AJ10" s="16">
-        <v>3.78</v>
+        <v>3.81</v>
       </c>
       <c r="AK10" s="16">
-        <v>20.18</v>
+        <v>20.329999999999998</v>
       </c>
       <c r="AL10" s="16">
-        <v>7.93</v>
+        <v>7.99</v>
       </c>
       <c r="AM10" s="16">
-        <v>1.8</v>
+        <v>1.81</v>
       </c>
       <c r="AN10" s="16">
-        <v>5.41</v>
+        <v>5.44</v>
       </c>
       <c r="AO10" s="16">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="AP10" s="16">
-        <v>1.26</v>
+        <v>0.54</v>
       </c>
       <c r="AQ10" s="16">
-        <v>41.98</v>
+        <v>42.29</v>
       </c>
       <c r="AR10" s="17">
-        <v>5.23</v>
+        <v>5.26</v>
       </c>
       <c r="AS10" s="15">
         <v>12.41</v>
@@ -2249,12 +2241,12 @@
         <v>74.209999999999994</v>
       </c>
     </row>
-    <row r="11" spans="1:47" ht="105" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -2273,7 +2265,7 @@
       <c r="Q11" s="26"/>
       <c r="R11" s="27"/>
       <c r="S11" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="T11" s="26"/>
       <c r="U11" s="26"/>
@@ -2285,12 +2277,12 @@
       <c r="AA11" s="26"/>
       <c r="AB11" s="27"/>
       <c r="AC11" s="25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AD11" s="26"/>
       <c r="AE11" s="27"/>
       <c r="AF11" s="25" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="AG11" s="26"/>
       <c r="AH11" s="27"/>
@@ -2565,7 +2557,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate NRW building evidence into Aachen OSM analysis
</commit_message>
<xml_diff>
--- a/districtgenerator/data/typdistrict_parameters.xlsx
+++ b/districtgenerator/data/typdistrict_parameters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ResearchArtifacts\districtgenerator\tmp\osm_nrw_adoption_20261030_v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B0F1B52-63FF-4FBF-B32B-00B08FFE0E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52F0C05-9253-4E9B-A98E-233C4240D3D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11835" yWindow="-16335" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -1050,16 +1050,16 @@
         <v>3.5</v>
       </c>
       <c r="AI2" s="13">
-        <v>40.909999999999997</v>
+        <v>14.29</v>
       </c>
       <c r="AJ2" s="19">
-        <v>0</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="AK2" s="19">
-        <v>13.64</v>
+        <v>16.329999999999998</v>
       </c>
       <c r="AL2" s="19">
-        <v>4.55</v>
+        <v>4.08</v>
       </c>
       <c r="AM2" s="19">
         <v>0</v>
@@ -1068,25 +1068,25 @@
         <v>0</v>
       </c>
       <c r="AO2" s="19">
-        <v>13.64</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="AP2" s="19">
-        <v>4.55</v>
+        <v>2.04</v>
       </c>
       <c r="AQ2" s="19">
-        <v>13.64</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="AR2" s="14">
-        <v>9.09</v>
+        <v>32.65</v>
       </c>
       <c r="AS2" s="13">
-        <v>13.21</v>
+        <v>11.86</v>
       </c>
       <c r="AT2" s="19">
-        <v>0</v>
+        <v>1.45</v>
       </c>
       <c r="AU2" s="14">
-        <v>86.79</v>
+        <v>86.68</v>
       </c>
     </row>
     <row r="3" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1194,43 +1194,43 @@
         <v>3</v>
       </c>
       <c r="AI3" s="13">
-        <v>13.56</v>
+        <v>12.06</v>
       </c>
       <c r="AJ3" s="19">
-        <v>10.17</v>
+        <v>11.35</v>
       </c>
       <c r="AK3" s="19">
-        <v>12.71</v>
+        <v>13.48</v>
       </c>
       <c r="AL3" s="19">
-        <v>8.4700000000000006</v>
+        <v>7.09</v>
       </c>
       <c r="AM3" s="19">
-        <v>0</v>
+        <v>1.06</v>
       </c>
       <c r="AN3" s="19">
-        <v>1.69</v>
+        <v>4.26</v>
       </c>
       <c r="AO3" s="19">
-        <v>3.39</v>
+        <v>2.84</v>
       </c>
       <c r="AP3" s="19">
-        <v>3.39</v>
+        <v>1.77</v>
       </c>
       <c r="AQ3" s="19">
-        <v>22.03</v>
+        <v>14.89</v>
       </c>
       <c r="AR3" s="14">
-        <v>24.58</v>
+        <v>31.21</v>
       </c>
       <c r="AS3" s="13">
-        <v>10.91</v>
+        <v>2.91</v>
       </c>
       <c r="AT3" s="19">
-        <v>0.95</v>
+        <v>2.13</v>
       </c>
       <c r="AU3" s="14">
-        <v>88.15</v>
+        <v>94.96</v>
       </c>
     </row>
     <row r="4" spans="1:47" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1338,43 +1338,43 @@
         <v>3.5</v>
       </c>
       <c r="AI4" s="13">
-        <v>8.57</v>
+        <v>10.95</v>
       </c>
       <c r="AJ4" s="19">
-        <v>17.71</v>
+        <v>20.8</v>
       </c>
       <c r="AK4" s="19">
-        <v>7.43</v>
+        <v>6.57</v>
       </c>
       <c r="AL4" s="19">
-        <v>6.29</v>
+        <v>4.38</v>
       </c>
       <c r="AM4" s="19">
-        <v>1.1399999999999999</v>
+        <v>0</v>
       </c>
       <c r="AN4" s="19">
-        <v>4.57</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="AO4" s="19">
-        <v>4</v>
+        <v>4.01</v>
       </c>
       <c r="AP4" s="19">
-        <v>1.71</v>
+        <v>5.1100000000000003</v>
       </c>
       <c r="AQ4" s="19">
-        <v>22.29</v>
+        <v>17.52</v>
       </c>
       <c r="AR4" s="14">
-        <v>26.29</v>
+        <v>28.1</v>
       </c>
       <c r="AS4" s="13">
-        <v>25.76</v>
+        <v>6.23</v>
       </c>
       <c r="AT4" s="19">
-        <v>1.08</v>
+        <v>2.63</v>
       </c>
       <c r="AU4" s="14">
-        <v>73.16</v>
+        <v>91.14</v>
       </c>
     </row>
     <row r="5" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1482,43 +1482,43 @@
         <v>3.5</v>
       </c>
       <c r="AI5" s="13">
-        <v>9.84</v>
+        <v>13.45</v>
       </c>
       <c r="AJ5" s="19">
-        <v>15.26</v>
+        <v>16.260000000000002</v>
       </c>
       <c r="AK5" s="19">
-        <v>9.44</v>
+        <v>8.44</v>
       </c>
       <c r="AL5" s="19">
-        <v>5.62</v>
+        <v>5.13</v>
       </c>
       <c r="AM5" s="19">
-        <v>6.63</v>
+        <v>1.59</v>
       </c>
       <c r="AN5" s="19">
-        <v>4.22</v>
+        <v>3.42</v>
       </c>
       <c r="AO5" s="19">
-        <v>2.81</v>
+        <v>1.47</v>
       </c>
       <c r="AP5" s="19">
-        <v>0.2</v>
+        <v>3.06</v>
       </c>
       <c r="AQ5" s="19">
-        <v>23.49</v>
+        <v>23.84</v>
       </c>
       <c r="AR5" s="14">
-        <v>22.49</v>
+        <v>23.35</v>
       </c>
       <c r="AS5" s="13">
-        <v>22.09</v>
+        <v>7.62</v>
       </c>
       <c r="AT5" s="19">
-        <v>1.1000000000000001</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="AU5" s="14">
-        <v>76.8</v>
+        <v>87.98</v>
       </c>
     </row>
     <row r="6" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1626,43 +1626,43 @@
         <v>3</v>
       </c>
       <c r="AI6" s="13">
-        <v>5.88</v>
+        <v>8.0299999999999994</v>
       </c>
       <c r="AJ6" s="19">
-        <v>17.97</v>
+        <v>13.08</v>
       </c>
       <c r="AK6" s="19">
-        <v>18.600000000000001</v>
+        <v>13.6</v>
       </c>
       <c r="AL6" s="19">
-        <v>8.11</v>
+        <v>5.96</v>
       </c>
       <c r="AM6" s="19">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="AN6" s="19">
-        <v>7.79</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="AO6" s="19">
-        <v>2.38</v>
+        <v>1.81</v>
       </c>
       <c r="AP6" s="19">
-        <v>1.1100000000000001</v>
+        <v>1.55</v>
       </c>
       <c r="AQ6" s="19">
-        <v>25.6</v>
+        <v>20.079999999999998</v>
       </c>
       <c r="AR6" s="14">
-        <v>12.56</v>
+        <v>31.35</v>
       </c>
       <c r="AS6" s="13">
-        <v>6.43</v>
+        <v>1.86</v>
       </c>
       <c r="AT6" s="19">
-        <v>0.56999999999999995</v>
+        <v>3.01</v>
       </c>
       <c r="AU6" s="14">
-        <v>93</v>
+        <v>95.13</v>
       </c>
     </row>
     <row r="7" spans="1:47" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1776,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="AK7" s="19">
-        <v>16.670000000000002</v>
+        <v>0</v>
       </c>
       <c r="AL7" s="19">
         <v>0</v>
@@ -1788,25 +1788,25 @@
         <v>0</v>
       </c>
       <c r="AO7" s="19">
-        <v>0</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="AP7" s="19">
         <v>0</v>
       </c>
       <c r="AQ7" s="19">
-        <v>33.33</v>
+        <v>26.09</v>
       </c>
       <c r="AR7" s="14">
-        <v>50</v>
+        <v>69.569999999999993</v>
       </c>
       <c r="AS7" s="13">
-        <v>22.86</v>
+        <v>17.829999999999998</v>
       </c>
       <c r="AT7" s="19">
-        <v>0</v>
+        <v>5.43</v>
       </c>
       <c r="AU7" s="14">
-        <v>77.14</v>
+        <v>76.739999999999995</v>
       </c>
     </row>
     <row r="8" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1914,43 +1914,43 @@
         <v>19</v>
       </c>
       <c r="AI8" s="13">
-        <v>11.39</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="AJ8" s="19">
-        <v>20.3</v>
+        <v>16.86</v>
       </c>
       <c r="AK8" s="19">
-        <v>7.43</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="AL8" s="19">
-        <v>2.97</v>
+        <v>2.91</v>
       </c>
       <c r="AM8" s="19">
-        <v>12.87</v>
+        <v>26.74</v>
       </c>
       <c r="AN8" s="19">
-        <v>5.45</v>
+        <v>5.81</v>
       </c>
       <c r="AO8" s="19">
-        <v>2.48</v>
+        <v>1.74</v>
       </c>
       <c r="AP8" s="19">
-        <v>2.97</v>
+        <v>4.07</v>
       </c>
       <c r="AQ8" s="19">
-        <v>12.87</v>
+        <v>16.86</v>
       </c>
       <c r="AR8" s="14">
-        <v>21.29</v>
+        <v>7.56</v>
       </c>
       <c r="AS8" s="13">
-        <v>30.3</v>
+        <v>18.61</v>
       </c>
       <c r="AT8" s="19">
-        <v>2.7</v>
+        <v>4.99</v>
       </c>
       <c r="AU8" s="14">
-        <v>67.010000000000005</v>
+        <v>76.400000000000006</v>
       </c>
     </row>
     <row r="9" spans="1:47" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2058,43 +2058,43 @@
         <v>6</v>
       </c>
       <c r="AI9" s="13">
-        <v>16.27</v>
+        <v>21.35</v>
       </c>
       <c r="AJ9" s="19">
-        <v>14.92</v>
+        <v>8.9</v>
       </c>
       <c r="AK9" s="19">
-        <v>9.15</v>
+        <v>8.19</v>
       </c>
       <c r="AL9" s="19">
-        <v>5.08</v>
+        <v>3.91</v>
       </c>
       <c r="AM9" s="19">
-        <v>7.46</v>
+        <v>7.83</v>
       </c>
       <c r="AN9" s="19">
-        <v>10.17</v>
+        <v>8.9</v>
       </c>
       <c r="AO9" s="19">
-        <v>1.69</v>
+        <v>1.42</v>
       </c>
       <c r="AP9" s="19">
-        <v>3.05</v>
+        <v>2.14</v>
       </c>
       <c r="AQ9" s="19">
-        <v>25.08</v>
+        <v>27.4</v>
       </c>
       <c r="AR9" s="14">
-        <v>7.12</v>
+        <v>9.9600000000000009</v>
       </c>
       <c r="AS9" s="13">
-        <v>19.88</v>
+        <v>15.42</v>
       </c>
       <c r="AT9" s="19">
-        <v>7.92</v>
+        <v>12.64</v>
       </c>
       <c r="AU9" s="14">
-        <v>72.2</v>
+        <v>71.95</v>
       </c>
     </row>
     <row r="10" spans="1:47" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2202,43 +2202,43 @@
         <v>6.5</v>
       </c>
       <c r="AI10" s="15">
-        <v>10.53</v>
+        <v>12.09</v>
       </c>
       <c r="AJ10" s="16">
-        <v>3.81</v>
+        <v>5.13</v>
       </c>
       <c r="AK10" s="16">
-        <v>20.329999999999998</v>
+        <v>19.54</v>
       </c>
       <c r="AL10" s="16">
-        <v>7.99</v>
+        <v>8.11</v>
       </c>
       <c r="AM10" s="16">
-        <v>1.81</v>
+        <v>1.82</v>
       </c>
       <c r="AN10" s="16">
-        <v>5.44</v>
+        <v>5.13</v>
       </c>
       <c r="AO10" s="16">
-        <v>2</v>
+        <v>2.48</v>
       </c>
       <c r="AP10" s="16">
-        <v>0.54</v>
+        <v>0.5</v>
       </c>
       <c r="AQ10" s="16">
-        <v>42.29</v>
+        <v>37.42</v>
       </c>
       <c r="AR10" s="17">
-        <v>5.26</v>
+        <v>7.78</v>
       </c>
       <c r="AS10" s="15">
-        <v>12.41</v>
+        <v>9.7799999999999994</v>
       </c>
       <c r="AT10" s="16">
-        <v>13.38</v>
+        <v>19.829999999999998</v>
       </c>
       <c r="AU10" s="17">
-        <v>74.209999999999994</v>
+        <v>70.39</v>
       </c>
     </row>
     <row r="11" spans="1:47" ht="105" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>